<commit_message>
update excel a bit
</commit_message>
<xml_diff>
--- a/src/excel_templates/purchase_request_template.xlsx
+++ b/src/excel_templates/purchase_request_template.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="24">
   <si>
     <t xml:space="preserve">Date: </t>
   </si>
@@ -77,6 +77,9 @@
   </si>
   <si>
     <t>Shipping</t>
+  </si>
+  <si>
+    <t>Total (CAD)</t>
   </si>
   <si>
     <t>Are you the Purchasor?</t>
@@ -1118,7 +1121,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18">
       <c r="A30" s="31" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B30" s="20"/>
       <c r="C30" s="4"/>
@@ -1129,7 +1132,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18">
       <c r="A31" s="32" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B31" s="33"/>
       <c r="C31" s="4"/>
@@ -1140,7 +1143,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18">
       <c r="A32" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B32" s="17"/>
       <c r="C32" s="4"/>
@@ -1151,7 +1154,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18">
       <c r="A33" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B33" s="17"/>
       <c r="C33" s="4"/>
@@ -1351,7 +1354,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18">
       <c r="A55" s="36" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B55" s="20"/>
       <c r="C55" s="26"/>
@@ -1398,7 +1401,7 @@
     <col min="7" max="7" style="39" width="13.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1435,7 +1438,7 @@
       <c r="F3" s="5"/>
       <c r="G3" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
@@ -1468,7 +1471,7 @@
       <c r="F6" s="5"/>
       <c r="G6" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="20.25">
       <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
@@ -1513,7 +1516,7 @@
         <v>15</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="1">
         <v>2</v>
       </c>
@@ -1524,7 +1527,7 @@
       <c r="F10" s="19"/>
       <c r="G10" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="1">
         <v>3</v>
       </c>
@@ -1712,7 +1715,7 @@
       <c r="C27" s="29"/>
       <c r="D27" s="29"/>
       <c r="E27" s="3" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F27" s="25">
         <v>0</v>
@@ -1739,7 +1742,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18">
       <c r="A30" s="31" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B30" s="20"/>
       <c r="C30" s="4"/>
@@ -1750,7 +1753,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18">
       <c r="A31" s="32" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B31" s="33"/>
       <c r="C31" s="4"/>
@@ -1761,7 +1764,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18">
       <c r="A32" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B32" s="17"/>
       <c r="C32" s="4"/>
@@ -1772,7 +1775,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18">
       <c r="A33" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B33" s="17"/>
       <c r="C33" s="4"/>
@@ -1972,7 +1975,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18">
       <c r="A55" s="36" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B55" s="20"/>
       <c r="C55" s="26"/>
@@ -2360,7 +2363,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18">
       <c r="A30" s="31" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B30" s="20"/>
       <c r="C30" s="4"/>
@@ -2371,7 +2374,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18">
       <c r="A31" s="32" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B31" s="33"/>
       <c r="C31" s="4"/>
@@ -2382,7 +2385,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18">
       <c r="A32" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B32" s="17"/>
       <c r="C32" s="4"/>
@@ -2393,7 +2396,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18">
       <c r="A33" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B33" s="17"/>
       <c r="C33" s="4"/>
@@ -2593,7 +2596,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18">
       <c r="A55" s="36" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B55" s="20"/>
       <c r="C55" s="26"/>
@@ -2981,7 +2984,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18">
       <c r="A30" s="31" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B30" s="20"/>
       <c r="C30" s="4"/>
@@ -2992,7 +2995,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18">
       <c r="A31" s="32" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B31" s="33"/>
       <c r="C31" s="4"/>
@@ -3003,7 +3006,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18">
       <c r="A32" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B32" s="17"/>
       <c r="C32" s="4"/>
@@ -3014,7 +3017,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18">
       <c r="A33" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B33" s="17"/>
       <c r="C33" s="4"/>
@@ -3214,7 +3217,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18">
       <c r="A55" s="36" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B55" s="20"/>
       <c r="C55" s="26"/>
@@ -3602,7 +3605,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18">
       <c r="A30" s="31" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B30" s="20"/>
       <c r="C30" s="4"/>
@@ -3613,7 +3616,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18">
       <c r="A31" s="32" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B31" s="33"/>
       <c r="C31" s="4"/>
@@ -3624,7 +3627,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18">
       <c r="A32" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B32" s="17"/>
       <c r="C32" s="4"/>
@@ -3635,7 +3638,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18">
       <c r="A33" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B33" s="17"/>
       <c r="C33" s="4"/>
@@ -3835,7 +3838,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18">
       <c r="A55" s="36" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B55" s="20"/>
       <c r="C55" s="26"/>
@@ -4223,7 +4226,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18">
       <c r="A30" s="31" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B30" s="20"/>
       <c r="C30" s="4"/>
@@ -4234,7 +4237,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18">
       <c r="A31" s="32" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B31" s="33"/>
       <c r="C31" s="4"/>
@@ -4245,7 +4248,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18">
       <c r="A32" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B32" s="17"/>
       <c r="C32" s="4"/>
@@ -4256,7 +4259,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18">
       <c r="A33" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B33" s="17"/>
       <c r="C33" s="4"/>
@@ -4456,7 +4459,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18">
       <c r="A55" s="36" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B55" s="20"/>
       <c r="C55" s="26"/>
@@ -4844,7 +4847,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18">
       <c r="A30" s="31" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B30" s="20"/>
       <c r="C30" s="4"/>
@@ -4855,7 +4858,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18">
       <c r="A31" s="32" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B31" s="33"/>
       <c r="C31" s="4"/>
@@ -4866,7 +4869,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18">
       <c r="A32" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B32" s="17"/>
       <c r="C32" s="4"/>
@@ -4877,7 +4880,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18">
       <c r="A33" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B33" s="17"/>
       <c r="C33" s="4"/>
@@ -5077,7 +5080,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18">
       <c r="A55" s="36" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B55" s="20"/>
       <c r="C55" s="26"/>
@@ -5465,7 +5468,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18">
       <c r="A30" s="31" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B30" s="20"/>
       <c r="C30" s="4"/>
@@ -5476,7 +5479,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18">
       <c r="A31" s="32" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B31" s="33"/>
       <c r="C31" s="4"/>
@@ -5487,7 +5490,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18">
       <c r="A32" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B32" s="17"/>
       <c r="C32" s="4"/>
@@ -5498,7 +5501,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18">
       <c r="A33" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B33" s="17"/>
       <c r="C33" s="4"/>
@@ -5698,7 +5701,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18">
       <c r="A55" s="36" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B55" s="20"/>
       <c r="C55" s="26"/>
@@ -6086,7 +6089,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18">
       <c r="A30" s="31" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B30" s="20"/>
       <c r="C30" s="4"/>
@@ -6097,7 +6100,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18">
       <c r="A31" s="32" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B31" s="33"/>
       <c r="C31" s="4"/>
@@ -6108,7 +6111,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18">
       <c r="A32" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B32" s="17"/>
       <c r="C32" s="4"/>
@@ -6119,7 +6122,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18">
       <c r="A33" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B33" s="17"/>
       <c r="C33" s="4"/>
@@ -6319,7 +6322,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18">
       <c r="A55" s="36" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B55" s="20"/>
       <c r="C55" s="26"/>
@@ -6707,7 +6710,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18">
       <c r="A30" s="31" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B30" s="20"/>
       <c r="C30" s="4"/>
@@ -6718,7 +6721,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18">
       <c r="A31" s="32" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B31" s="33"/>
       <c r="C31" s="4"/>
@@ -6729,7 +6732,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18">
       <c r="A32" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B32" s="17"/>
       <c r="C32" s="4"/>
@@ -6740,7 +6743,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18">
       <c r="A33" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B33" s="17"/>
       <c r="C33" s="4"/>
@@ -6940,7 +6943,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18">
       <c r="A55" s="36" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B55" s="20"/>
       <c r="C55" s="26"/>

</xml_diff>

<commit_message>
better refactor of data processing (#237)
</commit_message>
<xml_diff>
--- a/src/excel_templates/purchase_request_template.xlsx
+++ b/src/excel_templates/purchase_request_template.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="24">
   <si>
     <t xml:space="preserve">Date: </t>
   </si>
@@ -77,6 +77,9 @@
   </si>
   <si>
     <t>Shipping</t>
+  </si>
+  <si>
+    <t>Total (CAD)</t>
   </si>
   <si>
     <t>Are you the Purchasor?</t>
@@ -1118,7 +1121,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18">
       <c r="A30" s="31" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B30" s="20"/>
       <c r="C30" s="4"/>
@@ -1129,7 +1132,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18">
       <c r="A31" s="32" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B31" s="33"/>
       <c r="C31" s="4"/>
@@ -1140,7 +1143,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18">
       <c r="A32" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B32" s="17"/>
       <c r="C32" s="4"/>
@@ -1151,7 +1154,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18">
       <c r="A33" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B33" s="17"/>
       <c r="C33" s="4"/>
@@ -1351,7 +1354,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18">
       <c r="A55" s="36" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B55" s="20"/>
       <c r="C55" s="26"/>
@@ -1398,7 +1401,7 @@
     <col min="7" max="7" style="39" width="13.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1435,7 +1438,7 @@
       <c r="F3" s="5"/>
       <c r="G3" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
@@ -1468,7 +1471,7 @@
       <c r="F6" s="5"/>
       <c r="G6" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="20.25">
       <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
@@ -1513,7 +1516,7 @@
         <v>15</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="1">
         <v>2</v>
       </c>
@@ -1524,7 +1527,7 @@
       <c r="F10" s="19"/>
       <c r="G10" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="1">
         <v>3</v>
       </c>
@@ -1712,7 +1715,7 @@
       <c r="C27" s="29"/>
       <c r="D27" s="29"/>
       <c r="E27" s="3" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F27" s="25">
         <v>0</v>
@@ -1739,7 +1742,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18">
       <c r="A30" s="31" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B30" s="20"/>
       <c r="C30" s="4"/>
@@ -1750,7 +1753,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18">
       <c r="A31" s="32" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B31" s="33"/>
       <c r="C31" s="4"/>
@@ -1761,7 +1764,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18">
       <c r="A32" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B32" s="17"/>
       <c r="C32" s="4"/>
@@ -1772,7 +1775,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18">
       <c r="A33" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B33" s="17"/>
       <c r="C33" s="4"/>
@@ -1972,7 +1975,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18">
       <c r="A55" s="36" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B55" s="20"/>
       <c r="C55" s="26"/>
@@ -2360,7 +2363,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18">
       <c r="A30" s="31" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B30" s="20"/>
       <c r="C30" s="4"/>
@@ -2371,7 +2374,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18">
       <c r="A31" s="32" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B31" s="33"/>
       <c r="C31" s="4"/>
@@ -2382,7 +2385,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18">
       <c r="A32" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B32" s="17"/>
       <c r="C32" s="4"/>
@@ -2393,7 +2396,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18">
       <c r="A33" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B33" s="17"/>
       <c r="C33" s="4"/>
@@ -2593,7 +2596,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18">
       <c r="A55" s="36" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B55" s="20"/>
       <c r="C55" s="26"/>
@@ -2981,7 +2984,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18">
       <c r="A30" s="31" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B30" s="20"/>
       <c r="C30" s="4"/>
@@ -2992,7 +2995,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18">
       <c r="A31" s="32" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B31" s="33"/>
       <c r="C31" s="4"/>
@@ -3003,7 +3006,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18">
       <c r="A32" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B32" s="17"/>
       <c r="C32" s="4"/>
@@ -3014,7 +3017,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18">
       <c r="A33" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B33" s="17"/>
       <c r="C33" s="4"/>
@@ -3214,7 +3217,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18">
       <c r="A55" s="36" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B55" s="20"/>
       <c r="C55" s="26"/>
@@ -3602,7 +3605,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18">
       <c r="A30" s="31" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B30" s="20"/>
       <c r="C30" s="4"/>
@@ -3613,7 +3616,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18">
       <c r="A31" s="32" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B31" s="33"/>
       <c r="C31" s="4"/>
@@ -3624,7 +3627,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18">
       <c r="A32" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B32" s="17"/>
       <c r="C32" s="4"/>
@@ -3635,7 +3638,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18">
       <c r="A33" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B33" s="17"/>
       <c r="C33" s="4"/>
@@ -3835,7 +3838,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18">
       <c r="A55" s="36" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B55" s="20"/>
       <c r="C55" s="26"/>
@@ -4223,7 +4226,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18">
       <c r="A30" s="31" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B30" s="20"/>
       <c r="C30" s="4"/>
@@ -4234,7 +4237,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18">
       <c r="A31" s="32" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B31" s="33"/>
       <c r="C31" s="4"/>
@@ -4245,7 +4248,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18">
       <c r="A32" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B32" s="17"/>
       <c r="C32" s="4"/>
@@ -4256,7 +4259,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18">
       <c r="A33" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B33" s="17"/>
       <c r="C33" s="4"/>
@@ -4456,7 +4459,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18">
       <c r="A55" s="36" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B55" s="20"/>
       <c r="C55" s="26"/>
@@ -4844,7 +4847,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18">
       <c r="A30" s="31" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B30" s="20"/>
       <c r="C30" s="4"/>
@@ -4855,7 +4858,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18">
       <c r="A31" s="32" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B31" s="33"/>
       <c r="C31" s="4"/>
@@ -4866,7 +4869,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18">
       <c r="A32" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B32" s="17"/>
       <c r="C32" s="4"/>
@@ -4877,7 +4880,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18">
       <c r="A33" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B33" s="17"/>
       <c r="C33" s="4"/>
@@ -5077,7 +5080,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18">
       <c r="A55" s="36" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B55" s="20"/>
       <c r="C55" s="26"/>
@@ -5465,7 +5468,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18">
       <c r="A30" s="31" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B30" s="20"/>
       <c r="C30" s="4"/>
@@ -5476,7 +5479,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18">
       <c r="A31" s="32" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B31" s="33"/>
       <c r="C31" s="4"/>
@@ -5487,7 +5490,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18">
       <c r="A32" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B32" s="17"/>
       <c r="C32" s="4"/>
@@ -5498,7 +5501,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18">
       <c r="A33" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B33" s="17"/>
       <c r="C33" s="4"/>
@@ -5698,7 +5701,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18">
       <c r="A55" s="36" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B55" s="20"/>
       <c r="C55" s="26"/>
@@ -6086,7 +6089,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18">
       <c r="A30" s="31" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B30" s="20"/>
       <c r="C30" s="4"/>
@@ -6097,7 +6100,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18">
       <c r="A31" s="32" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B31" s="33"/>
       <c r="C31" s="4"/>
@@ -6108,7 +6111,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18">
       <c r="A32" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B32" s="17"/>
       <c r="C32" s="4"/>
@@ -6119,7 +6122,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18">
       <c r="A33" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B33" s="17"/>
       <c r="C33" s="4"/>
@@ -6319,7 +6322,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18">
       <c r="A55" s="36" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B55" s="20"/>
       <c r="C55" s="26"/>
@@ -6707,7 +6710,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18">
       <c r="A30" s="31" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B30" s="20"/>
       <c r="C30" s="4"/>
@@ -6718,7 +6721,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18">
       <c r="A31" s="32" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B31" s="33"/>
       <c r="C31" s="4"/>
@@ -6729,7 +6732,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18">
       <c r="A32" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B32" s="17"/>
       <c r="C32" s="4"/>
@@ -6740,7 +6743,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18">
       <c r="A33" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B33" s="17"/>
       <c r="C33" s="4"/>
@@ -6940,7 +6943,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18">
       <c r="A55" s="36" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B55" s="20"/>
       <c r="C55" s="26"/>

</xml_diff>